<commit_message>
fix: validate PostgreSQL demo stack
</commit_message>
<xml_diff>
--- a/assets/sample_outputs/funding_program_brief.xlsx
+++ b/assets/sample_outputs/funding_program_brief.xlsx
@@ -397,13 +397,13 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C2">
         <v>1</v>
       </c>
       <c r="D2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E2">
         <v>32184.26</v>
@@ -417,13 +417,13 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C3">
         <v>2</v>
       </c>
       <c r="D3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E3">
         <v>53111.34</v>
@@ -437,13 +437,13 @@
         <v>3</v>
       </c>
       <c r="B4">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C4">
         <v>3</v>
       </c>
       <c r="D4">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E4">
         <v>65066.94</v>
@@ -457,13 +457,13 @@
         <v>4</v>
       </c>
       <c r="B5">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C5">
         <v>4</v>
       </c>
       <c r="D5">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E5">
         <v>58303.44</v>
@@ -477,13 +477,13 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C6">
         <v>5</v>
       </c>
       <c r="D6">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E6">
         <v>29145.4</v>
@@ -497,13 +497,13 @@
         <v>6</v>
       </c>
       <c r="B7">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C7">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="D7">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E7">
         <v>60595.53</v>
@@ -517,13 +517,13 @@
         <v>7</v>
       </c>
       <c r="B8">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C8">
         <v>1</v>
       </c>
       <c r="D8">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E8">
         <v>11845.16</v>
@@ -537,13 +537,13 @@
         <v>8</v>
       </c>
       <c r="B9">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C9">
         <v>2</v>
       </c>
       <c r="D9">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E9">
         <v>43485.83</v>
@@ -557,13 +557,13 @@
         <v>9</v>
       </c>
       <c r="B10">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C10">
         <v>3</v>
       </c>
       <c r="D10">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E10">
         <v>18328.37</v>
@@ -577,13 +577,13 @@
         <v>10</v>
       </c>
       <c r="B11">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C11">
         <v>4</v>
       </c>
       <c r="D11">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E11">
         <v>28934.52</v>
@@ -597,13 +597,13 @@
         <v>11</v>
       </c>
       <c r="B12">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C12">
         <v>5</v>
       </c>
       <c r="D12">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E12">
         <v>79015.60000000001</v>
@@ -617,13 +617,13 @@
         <v>12</v>
       </c>
       <c r="B13">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="C13">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="D13">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E13">
         <v>26884.44</v>
@@ -637,13 +637,13 @@
         <v>13</v>
       </c>
       <c r="B14">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C14">
         <v>1</v>
       </c>
       <c r="D14">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E14">
         <v>87982.92</v>
@@ -657,13 +657,13 @@
         <v>14</v>
       </c>
       <c r="B15">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C15">
         <v>2</v>
       </c>
       <c r="D15">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E15">
         <v>90344.41</v>
@@ -677,13 +677,13 @@
         <v>15</v>
       </c>
       <c r="B16">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C16">
         <v>3</v>
       </c>
       <c r="D16">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E16">
         <v>22876.14</v>
@@ -697,13 +697,13 @@
         <v>16</v>
       </c>
       <c r="B17">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C17">
         <v>4</v>
       </c>
       <c r="D17">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E17">
         <v>11168.85</v>
@@ -717,13 +717,13 @@
         <v>17</v>
       </c>
       <c r="B18">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C18">
         <v>5</v>
       </c>
       <c r="D18">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E18">
         <v>34803.95</v>
@@ -737,13 +737,13 @@
         <v>18</v>
       </c>
       <c r="B19">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C19">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="D19">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E19">
         <v>94692.49000000001</v>
@@ -757,13 +757,13 @@
         <v>19</v>
       </c>
       <c r="B20">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C20">
         <v>1</v>
       </c>
       <c r="D20">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E20">
         <v>60304.33</v>
@@ -777,13 +777,13 @@
         <v>20</v>
       </c>
       <c r="B21">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C21">
         <v>2</v>
       </c>
       <c r="D21">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E21">
         <v>94922.03</v>
@@ -797,13 +797,13 @@
         <v>21</v>
       </c>
       <c r="B22">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C22">
         <v>3</v>
       </c>
       <c r="D22">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E22">
         <v>42552.1</v>
@@ -817,13 +817,13 @@
         <v>22</v>
       </c>
       <c r="B23">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C23">
         <v>4</v>
       </c>
       <c r="D23">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E23">
         <v>57881.15</v>
@@ -837,13 +837,13 @@
         <v>23</v>
       </c>
       <c r="B24">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C24">
         <v>5</v>
       </c>
       <c r="D24">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E24">
         <v>20190.58</v>
@@ -857,13 +857,13 @@
         <v>24</v>
       </c>
       <c r="B25">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="C25">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="D25">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E25">
         <v>12164.63</v>
@@ -877,13 +877,13 @@
         <v>25</v>
       </c>
       <c r="B26">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C26">
         <v>1</v>
       </c>
       <c r="D26">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E26">
         <v>53673</v>
@@ -897,13 +897,13 @@
         <v>26</v>
       </c>
       <c r="B27">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C27">
         <v>2</v>
       </c>
       <c r="D27">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E27">
         <v>75957.28</v>
@@ -917,13 +917,13 @@
         <v>27</v>
       </c>
       <c r="B28">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C28">
         <v>3</v>
       </c>
       <c r="D28">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E28">
         <v>83714.13</v>
@@ -937,13 +937,13 @@
         <v>28</v>
       </c>
       <c r="B29">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C29">
         <v>4</v>
       </c>
       <c r="D29">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E29">
         <v>80439.17</v>
@@ -957,13 +957,13 @@
         <v>29</v>
       </c>
       <c r="B30">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C30">
         <v>5</v>
       </c>
       <c r="D30">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E30">
         <v>61219.94</v>
@@ -977,13 +977,13 @@
         <v>30</v>
       </c>
       <c r="B31">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C31">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="D31">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E31">
         <v>30056.75</v>
@@ -997,13 +997,13 @@
         <v>31</v>
       </c>
       <c r="B32">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C32">
         <v>1</v>
       </c>
       <c r="D32">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E32">
         <v>53913.37</v>
@@ -1017,13 +1017,13 @@
         <v>32</v>
       </c>
       <c r="B33">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C33">
         <v>2</v>
       </c>
       <c r="D33">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E33">
         <v>52367.15</v>
@@ -1037,13 +1037,13 @@
         <v>33</v>
       </c>
       <c r="B34">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C34">
         <v>3</v>
       </c>
       <c r="D34">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E34">
         <v>57847.76</v>
@@ -1057,13 +1057,13 @@
         <v>34</v>
       </c>
       <c r="B35">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C35">
         <v>4</v>
       </c>
       <c r="D35">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E35">
         <v>72776.25999999999</v>
@@ -1077,13 +1077,13 @@
         <v>35</v>
       </c>
       <c r="B36">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C36">
         <v>5</v>
       </c>
       <c r="D36">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E36">
         <v>38562.14</v>
@@ -1097,13 +1097,13 @@
         <v>36</v>
       </c>
       <c r="B37">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="C37">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="D37">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E37">
         <v>29470.46</v>
@@ -1117,13 +1117,13 @@
         <v>37</v>
       </c>
       <c r="B38">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C38">
         <v>1</v>
       </c>
       <c r="D38">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E38">
         <v>78972.53</v>
@@ -1137,13 +1137,13 @@
         <v>38</v>
       </c>
       <c r="B39">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C39">
         <v>2</v>
       </c>
       <c r="D39">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E39">
         <v>15851.7</v>
@@ -1157,13 +1157,13 @@
         <v>39</v>
       </c>
       <c r="B40">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C40">
         <v>3</v>
       </c>
       <c r="D40">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E40">
         <v>28686.65</v>
@@ -1177,13 +1177,13 @@
         <v>40</v>
       </c>
       <c r="B41">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C41">
         <v>4</v>
       </c>
       <c r="D41">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E41">
         <v>85131.53999999999</v>
@@ -1197,13 +1197,13 @@
         <v>41</v>
       </c>
       <c r="B42">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C42">
         <v>5</v>
       </c>
       <c r="D42">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E42">
         <v>94784.63</v>
@@ -1217,13 +1217,13 @@
         <v>42</v>
       </c>
       <c r="B43">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C43">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="D43">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E43">
         <v>45917.33</v>
@@ -1237,13 +1237,13 @@
         <v>43</v>
       </c>
       <c r="B44">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C44">
         <v>1</v>
       </c>
       <c r="D44">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E44">
         <v>72283.92999999999</v>
@@ -1257,13 +1257,13 @@
         <v>44</v>
       </c>
       <c r="B45">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C45">
         <v>2</v>
       </c>
       <c r="D45">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E45">
         <v>23542.41</v>
@@ -1277,13 +1277,13 @@
         <v>45</v>
       </c>
       <c r="B46">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C46">
         <v>3</v>
       </c>
       <c r="D46">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E46">
         <v>13069.95</v>
@@ -1297,13 +1297,13 @@
         <v>46</v>
       </c>
       <c r="B47">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C47">
         <v>4</v>
       </c>
       <c r="D47">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E47">
         <v>68453.42</v>
@@ -1317,13 +1317,13 @@
         <v>47</v>
       </c>
       <c r="B48">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C48">
         <v>5</v>
       </c>
       <c r="D48">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E48">
         <v>56161.26</v>
@@ -1337,13 +1337,13 @@
         <v>48</v>
       </c>
       <c r="B49">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="C49">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="D49">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E49">
         <v>36514.77</v>
@@ -1357,13 +1357,13 @@
         <v>49</v>
       </c>
       <c r="B50">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C50">
         <v>1</v>
       </c>
       <c r="D50">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E50">
         <v>38215.61</v>
@@ -1377,13 +1377,13 @@
         <v>50</v>
       </c>
       <c r="B51">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C51">
         <v>2</v>
       </c>
       <c r="D51">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E51">
         <v>10231.39</v>
@@ -1397,13 +1397,13 @@
         <v>51</v>
       </c>
       <c r="B52">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C52">
         <v>3</v>
       </c>
       <c r="D52">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E52">
         <v>47198.69</v>
@@ -1417,13 +1417,13 @@
         <v>52</v>
       </c>
       <c r="B53">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C53">
         <v>4</v>
       </c>
       <c r="D53">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E53">
         <v>91662.14999999999</v>
@@ -1437,13 +1437,13 @@
         <v>53</v>
       </c>
       <c r="B54">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C54">
         <v>5</v>
       </c>
       <c r="D54">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E54">
         <v>55580.64</v>
@@ -1457,13 +1457,13 @@
         <v>54</v>
       </c>
       <c r="B55">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C55">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="D55">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E55">
         <v>30866.18</v>
@@ -1477,13 +1477,13 @@
         <v>55</v>
       </c>
       <c r="B56">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C56">
         <v>1</v>
       </c>
       <c r="D56">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E56">
         <v>19766.4</v>
@@ -1497,13 +1497,13 @@
         <v>56</v>
       </c>
       <c r="B57">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C57">
         <v>2</v>
       </c>
       <c r="D57">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E57">
         <v>87809.94</v>
@@ -1517,13 +1517,13 @@
         <v>57</v>
       </c>
       <c r="B58">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C58">
         <v>3</v>
       </c>
       <c r="D58">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E58">
         <v>46080.42</v>
@@ -1537,13 +1537,13 @@
         <v>58</v>
       </c>
       <c r="B59">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C59">
         <v>4</v>
       </c>
       <c r="D59">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E59">
         <v>54698.73</v>
@@ -1557,13 +1557,13 @@
         <v>59</v>
       </c>
       <c r="B60">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C60">
         <v>5</v>
       </c>
       <c r="D60">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E60">
         <v>15816.24</v>
@@ -1577,13 +1577,13 @@
         <v>60</v>
       </c>
       <c r="B61">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="C61">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="D61">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E61">
         <v>66916.25</v>
@@ -1597,13 +1597,13 @@
         <v>61</v>
       </c>
       <c r="B62">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C62">
         <v>1</v>
       </c>
       <c r="D62">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E62">
         <v>33466.8</v>
@@ -1617,13 +1617,13 @@
         <v>62</v>
       </c>
       <c r="B63">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C63">
         <v>2</v>
       </c>
       <c r="D63">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E63">
         <v>75445.53999999999</v>
@@ -1637,13 +1637,13 @@
         <v>63</v>
       </c>
       <c r="B64">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C64">
         <v>3</v>
       </c>
       <c r="D64">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E64">
         <v>41127.61</v>
@@ -1657,13 +1657,13 @@
         <v>64</v>
       </c>
       <c r="B65">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C65">
         <v>4</v>
       </c>
       <c r="D65">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E65">
         <v>85767.64999999999</v>
@@ -1677,13 +1677,13 @@
         <v>65</v>
       </c>
       <c r="B66">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C66">
         <v>5</v>
       </c>
       <c r="D66">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E66">
         <v>82918.35000000001</v>
@@ -1697,13 +1697,13 @@
         <v>66</v>
       </c>
       <c r="B67">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C67">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="D67">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E67">
         <v>54547.92</v>
@@ -1717,13 +1717,13 @@
         <v>67</v>
       </c>
       <c r="B68">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C68">
         <v>1</v>
       </c>
       <c r="D68">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E68">
         <v>18266.88</v>
@@ -1737,13 +1737,13 @@
         <v>68</v>
       </c>
       <c r="B69">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C69">
         <v>2</v>
       </c>
       <c r="D69">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E69">
         <v>65159.92</v>
@@ -1757,13 +1757,13 @@
         <v>69</v>
       </c>
       <c r="B70">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C70">
         <v>3</v>
       </c>
       <c r="D70">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E70">
         <v>94056.14</v>
@@ -1777,13 +1777,13 @@
         <v>70</v>
       </c>
       <c r="B71">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C71">
         <v>4</v>
       </c>
       <c r="D71">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E71">
         <v>65069.79</v>
@@ -1797,13 +1797,13 @@
         <v>71</v>
       </c>
       <c r="B72">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C72">
         <v>5</v>
       </c>
       <c r="D72">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E72">
         <v>49901.3</v>
@@ -1817,13 +1817,13 @@
         <v>72</v>
       </c>
       <c r="B73">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="C73">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="D73">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E73">
         <v>51372.56</v>
@@ -1837,13 +1837,13 @@
         <v>73</v>
       </c>
       <c r="B74">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C74">
         <v>1</v>
       </c>
       <c r="D74">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E74">
         <v>70803.05</v>
@@ -1857,13 +1857,13 @@
         <v>74</v>
       </c>
       <c r="B75">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C75">
         <v>2</v>
       </c>
       <c r="D75">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E75">
         <v>43176.57</v>
@@ -1877,13 +1877,13 @@
         <v>75</v>
       </c>
       <c r="B76">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C76">
         <v>3</v>
       </c>
       <c r="D76">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E76">
         <v>57874.71</v>
@@ -1897,13 +1897,13 @@
         <v>76</v>
       </c>
       <c r="B77">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C77">
         <v>4</v>
       </c>
       <c r="D77">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E77">
         <v>88506.56</v>
@@ -1917,13 +1917,13 @@
         <v>77</v>
       </c>
       <c r="B78">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C78">
         <v>5</v>
       </c>
       <c r="D78">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="E78">
         <v>16520.49</v>
@@ -1937,13 +1937,13 @@
         <v>78</v>
       </c>
       <c r="B79">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C79">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="D79">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E79">
         <v>19292.35</v>
@@ -1957,13 +1957,13 @@
         <v>79</v>
       </c>
       <c r="B80">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C80">
         <v>1</v>
       </c>
       <c r="D80">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E80">
         <v>47382.12</v>
@@ -1977,13 +1977,13 @@
         <v>80</v>
       </c>
       <c r="B81">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C81">
         <v>2</v>
       </c>
       <c r="D81">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E81">
         <v>49378.75</v>
@@ -1997,13 +1997,13 @@
         <v>81</v>
       </c>
       <c r="B82">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C82">
         <v>3</v>
       </c>
       <c r="D82">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="E82">
         <v>62178.01</v>
@@ -2017,13 +2017,13 @@
         <v>82</v>
       </c>
       <c r="B83">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C83">
         <v>4</v>
       </c>
       <c r="D83">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E83">
         <v>31014.62</v>
@@ -2037,13 +2037,13 @@
         <v>83</v>
       </c>
       <c r="B84">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C84">
         <v>5</v>
       </c>
       <c r="D84">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E84">
         <v>82051.22</v>
@@ -2057,13 +2057,13 @@
         <v>84</v>
       </c>
       <c r="B85">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="C85">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="D85">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="E85">
         <v>18818.72</v>
@@ -2077,13 +2077,13 @@
         <v>85</v>
       </c>
       <c r="B86">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C86">
         <v>1</v>
       </c>
       <c r="D86">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="E86">
         <v>22845.57</v>
@@ -2097,13 +2097,13 @@
         <v>86</v>
       </c>
       <c r="B87">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C87">
         <v>2</v>
       </c>
       <c r="D87">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E87">
         <v>78058.14999999999</v>
@@ -2117,13 +2117,13 @@
         <v>87</v>
       </c>
       <c r="B88">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C88">
         <v>3</v>
       </c>
       <c r="D88">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E88">
         <v>60243.5</v>
@@ -2137,13 +2137,13 @@
         <v>88</v>
       </c>
       <c r="B89">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C89">
         <v>4</v>
       </c>
       <c r="D89">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="E89">
         <v>23702.32</v>
@@ -2157,13 +2157,13 @@
         <v>89</v>
       </c>
       <c r="B90">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C90">
         <v>5</v>
       </c>
       <c r="D90">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="E90">
         <v>64509.6</v>
@@ -2177,13 +2177,13 @@
         <v>90</v>
       </c>
       <c r="B91">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C91">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="D91">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="E91">
         <v>66007.86</v>
@@ -2197,13 +2197,13 @@
         <v>91</v>
       </c>
       <c r="B92">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C92">
         <v>1</v>
       </c>
       <c r="D92">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E92">
         <v>70247.56</v>
@@ -2217,13 +2217,13 @@
         <v>92</v>
       </c>
       <c r="B93">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C93">
         <v>2</v>
       </c>
       <c r="D93">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E93">
         <v>42116.81</v>
@@ -2237,13 +2237,13 @@
         <v>93</v>
       </c>
       <c r="B94">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C94">
         <v>3</v>
       </c>
       <c r="D94">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E94">
         <v>57318.84</v>
@@ -2257,13 +2257,13 @@
         <v>94</v>
       </c>
       <c r="B95">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C95">
         <v>4</v>
       </c>
       <c r="D95">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="E95">
         <v>82086.31</v>
@@ -2277,13 +2277,13 @@
         <v>95</v>
       </c>
       <c r="B96">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C96">
         <v>5</v>
       </c>
       <c r="D96">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E96">
         <v>66317.39999999999</v>
@@ -2297,13 +2297,13 @@
         <v>96</v>
       </c>
       <c r="B97">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="C97">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="D97">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E97">
         <v>47715.76</v>

</xml_diff>